<commit_message>
Interaction modification from main
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/data_format_1.xlsx
+++ b/src/test/resources/testdata/data_format_1.xlsx
@@ -527,12 +527,6 @@
     <t>22-08-2025</t>
   </si>
   <si>
-    <t>Interaction Name</t>
-  </si>
-  <si>
-    <t>Interaction ID</t>
-  </si>
-  <si>
     <t>DEMO   - McqInteraction</t>
   </si>
   <si>
@@ -669,6 +663,12 @@
   </si>
   <si>
     <t>practice test</t>
+  </si>
+  <si>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>Interaction Type</t>
   </si>
 </sst>
 </file>
@@ -1161,11 +1161,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="16" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B1" s="16" t="s">
         <v>1</v>
@@ -1186,45 +1186,45 @@
         <v>6</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="I1" s="16" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="J1" s="16" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="19" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C2" s="19" t="s">
         <v>98</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E2" s="16">
         <v>1234</v>
       </c>
       <c r="F2" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="G2" s="17" t="s">
+        <v>173</v>
+      </c>
+      <c r="H2" s="17" t="s">
         <v>174</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="I2" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="J2" s="17" t="s">
         <v>176</v>
-      </c>
-      <c r="I2" s="17" t="s">
-        <v>177</v>
-      </c>
-      <c r="J2" s="17" t="s">
-        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -1238,18 +1238,18 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>61</v>
       </c>
@@ -1263,7 +1263,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>86</v>
       </c>
@@ -1295,16 +1295,16 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="14.28515625" customWidth="1"/>
-    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="14.26953125" customWidth="1"/>
+    <col min="4" max="4" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>61</v>
       </c>
@@ -1324,7 +1324,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>86</v>
       </c>
@@ -1352,18 +1352,18 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="12.5703125" customWidth="1"/>
-    <col min="7" max="7" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="12.54296875" customWidth="1"/>
+    <col min="7" max="7" width="25.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="32.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>61</v>
       </c>
@@ -1392,7 +1392,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>86</v>
       </c>
@@ -1429,25 +1429,25 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5703125" customWidth="1"/>
-    <col min="7" max="7" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.85546875" customWidth="1"/>
-    <col min="9" max="9" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.54296875" customWidth="1"/>
+    <col min="7" max="7" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.81640625" customWidth="1"/>
+    <col min="9" max="9" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="32.453125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="26" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="24.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="23.26953125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>61</v>
       </c>
@@ -1491,7 +1491,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>113</v>
       </c>
@@ -1546,23 +1546,23 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:X2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5703125" customWidth="1"/>
-    <col min="7" max="7" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.85546875" customWidth="1"/>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.54296875" customWidth="1"/>
+    <col min="7" max="7" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.81640625" customWidth="1"/>
     <col min="9" max="9" width="29" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="38.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>61</v>
       </c>
@@ -1600,7 +1600,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>60</v>
       </c>
@@ -1659,18 +1659,18 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="22" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.1796875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="26.28515625" customWidth="1"/>
-    <col min="12" max="12" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="26.26953125" customWidth="1"/>
+    <col min="12" max="12" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>24</v>
       </c>
@@ -1711,7 +1711,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>56</v>
       </c>
@@ -1758,19 +1758,19 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.54296875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="46.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="46.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>57</v>
       </c>
@@ -1793,7 +1793,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>130</v>
       </c>
@@ -1826,15 +1826,15 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="46.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="46.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>57</v>
       </c>
@@ -1848,7 +1848,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>130</v>
       </c>
@@ -1872,21 +1872,21 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="38.453125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="32" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.453125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="20" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>57</v>
       </c>
@@ -1921,7 +1921,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>130</v>
       </c>
@@ -1969,17 +1969,17 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" customWidth="1"/>
+    <col min="3" max="3" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>57</v>
       </c>
@@ -2002,7 +2002,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>130</v>
       </c>
@@ -2036,17 +2036,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:S2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="18.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2072,18 +2072,18 @@
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>98</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E2">
         <v>1234</v>
@@ -2095,7 +2095,7 @@
         <v>45</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
@@ -2123,22 +2123,22 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.5703125" customWidth="1"/>
-    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.54296875" customWidth="1"/>
+    <col min="5" max="5" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>57</v>
       </c>
@@ -2173,7 +2173,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>130</v>
       </c>
@@ -2216,11 +2216,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="16" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B1" s="16" t="s">
         <v>1</v>
@@ -2244,30 +2244,30 @@
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="19" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C2" s="19" t="s">
         <v>98</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="E2" s="16">
         <v>1234</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G2" s="21" t="s">
         <v>6</v>
       </c>
       <c r="H2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -2281,11 +2281,11 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="16" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B1" s="16" t="s">
         <v>1</v>
@@ -2306,27 +2306,27 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="19" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C2" s="19" t="s">
         <v>98</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="E2" s="16">
         <v>1234</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="G2" s="18" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -2340,16 +2340,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="47.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="47.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="18.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>25</v>
       </c>
@@ -2357,24 +2357,24 @@
         <v>46</v>
       </c>
       <c r="C1" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>121</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D2" s="7"/>
       <c r="F2" s="3"/>
       <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C3" s="9"/>
     </row>
   </sheetData>
@@ -2386,28 +2386,28 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:W2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.28515625" customWidth="1"/>
-    <col min="4" max="4" width="20.85546875" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" customWidth="1"/>
-    <col min="7" max="7" width="34.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.5703125" customWidth="1"/>
-    <col min="9" max="9" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5703125" customWidth="1"/>
-    <col min="11" max="11" width="13.85546875" customWidth="1"/>
-    <col min="12" max="12" width="6.5703125" customWidth="1"/>
-    <col min="14" max="14" width="4.42578125" customWidth="1"/>
-    <col min="15" max="15" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19.140625" customWidth="1"/>
-    <col min="17" max="17" width="20.5703125" customWidth="1"/>
-    <col min="18" max="18" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" customWidth="1"/>
-    <col min="20" max="20" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.26953125" customWidth="1"/>
+    <col min="4" max="4" width="20.81640625" customWidth="1"/>
+    <col min="5" max="5" width="10.81640625" customWidth="1"/>
+    <col min="7" max="7" width="34.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.54296875" customWidth="1"/>
+    <col min="9" max="9" width="23.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.54296875" customWidth="1"/>
+    <col min="11" max="11" width="13.81640625" customWidth="1"/>
+    <col min="12" max="12" width="6.54296875" customWidth="1"/>
+    <col min="14" max="14" width="4.453125" customWidth="1"/>
+    <col min="15" max="15" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.1796875" customWidth="1"/>
+    <col min="17" max="17" width="20.54296875" customWidth="1"/>
+    <col min="18" max="18" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.81640625" customWidth="1"/>
+    <col min="20" max="20" width="20.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2463,13 +2463,13 @@
         <v>17</v>
       </c>
       <c r="S1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="T1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>119</v>
       </c>
@@ -2480,7 +2480,7 @@
         <v>98</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="E2" s="12">
         <v>9876543211</v>
@@ -2504,7 +2504,7 @@
         <v>2025</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
@@ -2521,7 +2521,7 @@
         <v>19</v>
       </c>
       <c r="S2" s="12" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="T2">
         <v>1234</v>
@@ -2544,25 +2544,25 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Y2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>57</v>
       </c>
       <c r="B1" t="s">
-        <v>165</v>
+        <v>210</v>
       </c>
       <c r="C1" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>130</v>
       </c>
@@ -2570,7 +2570,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -2601,9 +2601,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="16" t="s">
         <v>25</v>
       </c>
@@ -2611,66 +2611,66 @@
         <v>24</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D1" s="16" t="s">
         <v>46</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="G1" s="16" t="s">
         <v>29</v>
       </c>
       <c r="H1" s="16" t="s">
+        <v>198</v>
+      </c>
+      <c r="I1" s="16" t="s">
+        <v>199</v>
+      </c>
+      <c r="J1" s="16" t="s">
         <v>200</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="K1" s="16" t="s">
         <v>201</v>
       </c>
-      <c r="J1" s="16" t="s">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" s="17" t="s">
         <v>202</v>
       </c>
-      <c r="K1" s="16" t="s">
+      <c r="B2" s="17" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="C2" s="17" t="s">
         <v>204</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="D2" t="s">
         <v>205</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="E2" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" s="20" t="s">
         <v>207</v>
-      </c>
-      <c r="E2" s="16" t="s">
-        <v>208</v>
-      </c>
-      <c r="F2" s="20" t="s">
-        <v>209</v>
       </c>
       <c r="G2" s="18" t="s">
         <v>112</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="I2" s="17" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="J2" s="17" t="s">
+        <v>207</v>
+      </c>
+      <c r="K2" s="17" t="s">
         <v>209</v>
-      </c>
-      <c r="K2" s="17" t="s">
-        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -2681,19 +2681,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:S2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="38.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="38.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>24</v>
       </c>
@@ -2740,7 +2740,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>85</v>
       </c>

</xml_diff>